<commit_message>
Enforce ID-based LINDAS URI minting
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_AreaMgmt_v0.5.0.xlsx
+++ b/templates/Strukturvorlage_AreaMgmt_v0.5.0.xlsx
@@ -11259,7 +11259,11 @@
       <c r="F7" s="87" t="n"/>
       <c r="G7" s="130" t="n"/>
       <c r="H7" s="109" t="n"/>
-      <c r="I7" s="86" t="n"/>
+      <c r="I7" s="86" t="inlineStr">
+        <is>
+          <t>elevation</t>
+        </is>
+      </c>
       <c r="J7" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010000</t>
@@ -11275,13 +11279,15 @@
           <t>Räumliche Struktur</t>
         </is>
       </c>
-      <c r="M7" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K7,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N7" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K7,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="M7" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N7" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O7" s="87" t="inlineStr">
         <is>
@@ -11379,7 +11385,11 @@
       <c r="F8" s="87" t="n"/>
       <c r="G8" s="130" t="n"/>
       <c r="H8" s="109" t="n"/>
-      <c r="I8" s="86" t="n"/>
+      <c r="I8" s="86" t="inlineStr">
+        <is>
+          <t>site-area</t>
+        </is>
+      </c>
       <c r="J8" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010001</t>
@@ -11390,17 +11400,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L8" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K8,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K8,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N8" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K8,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L8" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M8" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N8" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O8" s="87" t="inlineStr">
         <is>
@@ -11498,7 +11511,11 @@
       <c r="F9" s="87" t="n"/>
       <c r="G9" s="130" t="n"/>
       <c r="H9" s="109" t="n"/>
-      <c r="I9" s="86" t="n"/>
+      <c r="I9" s="86" t="inlineStr">
+        <is>
+          <t>surrounding-area</t>
+        </is>
+      </c>
       <c r="J9" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010002</t>
@@ -11509,17 +11526,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L9" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K9,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K9,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N9" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K9,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L9" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M9" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N9" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O9" s="87" t="inlineStr">
         <is>
@@ -11625,7 +11645,11 @@
       <c r="F10" s="87" t="n"/>
       <c r="G10" s="130" t="n"/>
       <c r="H10" s="109" t="n"/>
-      <c r="I10" s="86" t="n"/>
+      <c r="I10" s="86" t="inlineStr">
+        <is>
+          <t>gross-floor-area</t>
+        </is>
+      </c>
       <c r="J10" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010003</t>
@@ -11636,17 +11660,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L10" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K10,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K10,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N10" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K10,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L10" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M10" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N10" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O10" s="91" t="inlineStr">
         <is>
@@ -11752,7 +11779,11 @@
       <c r="F11" s="87" t="n"/>
       <c r="G11" s="130" t="n"/>
       <c r="H11" s="109" t="n"/>
-      <c r="I11" s="86" t="n"/>
+      <c r="I11" s="86" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
       <c r="J11" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010004</t>
@@ -11763,17 +11794,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L11" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K11,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K11,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N11" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K11,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L11" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M11" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N11" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O11" s="87" t="inlineStr">
         <is>
@@ -11875,7 +11909,11 @@
       <c r="F12" s="87" t="n"/>
       <c r="G12" s="130" t="n"/>
       <c r="H12" s="109" t="n"/>
-      <c r="I12" s="86" t="n"/>
+      <c r="I12" s="86" t="inlineStr">
+        <is>
+          <t>external-room</t>
+        </is>
+      </c>
       <c r="J12" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010005</t>
@@ -11886,17 +11924,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L12" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K12,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K12,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K12,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L12" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M12" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N12" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O12" s="91" t="inlineStr">
         <is>
@@ -12002,7 +12043,11 @@
       <c r="F13" s="87" t="n"/>
       <c r="G13" s="130" t="n"/>
       <c r="H13" s="109" t="n"/>
-      <c r="I13" s="86" t="n"/>
+      <c r="I13" s="86" t="inlineStr">
+        <is>
+          <t>parking-space</t>
+        </is>
+      </c>
       <c r="J13" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010006</t>
@@ -12013,17 +12058,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L13" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K13,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K13,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K13,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L13" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M13" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N13" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O13" s="87" t="inlineStr">
         <is>
@@ -12129,7 +12177,11 @@
       <c r="F14" s="87" t="n"/>
       <c r="G14" s="130" t="n"/>
       <c r="H14" s="109" t="n"/>
-      <c r="I14" s="86" t="n"/>
+      <c r="I14" s="86" t="inlineStr">
+        <is>
+          <t>rentable-area</t>
+        </is>
+      </c>
       <c r="J14" s="87" t="inlineStr">
         <is>
           <t>IFMA_C_31010007</t>
@@ -12140,17 +12192,20 @@
           <t>Spatial structure</t>
         </is>
       </c>
-      <c r="L14" s="120">
-        <f>IFERROR(INDEX(Rules!$B:$B,MATCH(K14,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="120">
-        <f>IFERROR(INDEX(Rules!$C:$C,MATCH(K14,Rules!$A:$A,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N14" s="120">
-        <f>IFERROR(INDEX(Rules!$D:$D,MATCH(K14,Rules!$A:$A,0)),"")</f>
-        <v/>
+      <c r="L14" s="120" t="inlineStr">
+        <is>
+          <t>Räumliche Struktur</t>
+        </is>
+      </c>
+      <c r="M14" s="120" t="inlineStr">
+        <is>
+          <t>Structure spatiale</t>
+        </is>
+      </c>
+      <c r="N14" s="120" t="inlineStr">
+        <is>
+          <t>Struttura spaziale</t>
+        </is>
       </c>
       <c r="O14" s="87" t="inlineStr">
         <is>
@@ -13801,7 +13856,11 @@
       <c r="A7" s="117" t="n"/>
       <c r="C7" s="117" t="n"/>
       <c r="D7" s="119" t="n"/>
-      <c r="E7" s="86" t="n"/>
+      <c r="E7" s="86" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
       <c r="F7" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020002</t>
@@ -13812,17 +13871,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H7" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G7,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G7,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G7,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H7" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I7" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J7" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K7" s="110" t="inlineStr">
         <is>
@@ -13907,7 +13969,11 @@
       <c r="A8" s="117" t="n"/>
       <c r="C8" s="117" t="n"/>
       <c r="D8" s="119" t="n"/>
-      <c r="E8" s="86" t="n"/>
+      <c r="E8" s="86" t="inlineStr">
+        <is>
+          <t>longname</t>
+        </is>
+      </c>
       <c r="F8" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020003</t>
@@ -13918,17 +13984,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H8" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G8,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G8,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G8,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H8" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I8" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J8" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K8" s="110" t="inlineStr">
         <is>
@@ -14013,7 +14082,11 @@
       <c r="A9" s="117" t="n"/>
       <c r="C9" s="117" t="n"/>
       <c r="D9" s="119" t="n"/>
-      <c r="E9" s="86" t="n"/>
+      <c r="E9" s="86" t="inlineStr">
+        <is>
+          <t>sia-416-2003</t>
+        </is>
+      </c>
       <c r="F9" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020004</t>
@@ -14024,17 +14097,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H9" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G9,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G9,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G9,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H9" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I9" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J9" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K9" s="110" t="inlineStr">
         <is>
@@ -14123,7 +14199,11 @@
       <c r="A10" s="117" t="n"/>
       <c r="C10" s="117" t="n"/>
       <c r="D10" s="119" t="n"/>
-      <c r="E10" s="86" t="n"/>
+      <c r="E10" s="86" t="inlineStr">
+        <is>
+          <t>sia-380-2015</t>
+        </is>
+      </c>
       <c r="F10" s="110" t="inlineStr">
         <is>
           <t>IFMA_P_31020007</t>
@@ -14134,17 +14214,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H10" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G10,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G10,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G10,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H10" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I10" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J10" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K10" s="110" t="inlineStr">
         <is>
@@ -14233,7 +14316,11 @@
       <c r="A11" s="117" t="n"/>
       <c r="C11" s="117" t="n"/>
       <c r="D11" s="119" t="n"/>
-      <c r="E11" s="86" t="n"/>
+      <c r="E11" s="86" t="inlineStr">
+        <is>
+          <t>sia-2024-2021</t>
+        </is>
+      </c>
       <c r="F11" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020008</t>
@@ -14244,17 +14331,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H11" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G11,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I11" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G11,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G11,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H11" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I11" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J11" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K11" s="110" t="inlineStr">
         <is>
@@ -14343,7 +14433,11 @@
       <c r="A12" s="117" t="n"/>
       <c r="C12" s="117" t="n"/>
       <c r="D12" s="119" t="n"/>
-      <c r="E12" s="86" t="n"/>
+      <c r="E12" s="86" t="inlineStr">
+        <is>
+          <t>sia-d0615-2000</t>
+        </is>
+      </c>
       <c r="F12" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020010</t>
@@ -14354,17 +14448,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H12" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G12,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G12,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G12,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H12" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I12" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J12" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K12" s="110" t="inlineStr">
         <is>
@@ -14453,7 +14550,11 @@
       <c r="A13" s="117" t="n"/>
       <c r="C13" s="117" t="n"/>
       <c r="D13" s="119" t="n"/>
-      <c r="E13" s="86" t="n"/>
+      <c r="E13" s="86" t="inlineStr">
+        <is>
+          <t>programuse</t>
+        </is>
+      </c>
       <c r="F13" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020012</t>
@@ -14464,17 +14565,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H13" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G13,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G13,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G13,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H13" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I13" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J13" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K13" s="110" t="inlineStr">
         <is>
@@ -14563,7 +14667,11 @@
       <c r="A14" s="117" t="n"/>
       <c r="C14" s="117" t="n"/>
       <c r="D14" s="119" t="n"/>
-      <c r="E14" s="86" t="n"/>
+      <c r="E14" s="86" t="inlineStr">
+        <is>
+          <t>roomtype</t>
+        </is>
+      </c>
       <c r="F14" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020013</t>
@@ -14574,17 +14682,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H14" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G14,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G14,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G14,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H14" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I14" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J14" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K14" s="110" t="inlineStr">
         <is>
@@ -14673,7 +14784,11 @@
       <c r="A15" s="117" t="n"/>
       <c r="C15" s="117" t="n"/>
       <c r="D15" s="119" t="n"/>
-      <c r="E15" s="86" t="n"/>
+      <c r="E15" s="86" t="inlineStr">
+        <is>
+          <t>unittype</t>
+        </is>
+      </c>
       <c r="F15" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020014</t>
@@ -14684,17 +14799,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H15" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G15,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G15,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G15,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H15" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I15" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J15" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K15" s="110" t="inlineStr">
         <is>
@@ -14784,7 +14902,11 @@
       <c r="A16" s="117" t="n"/>
       <c r="C16" s="117" t="n"/>
       <c r="D16" s="119" t="n"/>
-      <c r="E16" s="86" t="n"/>
+      <c r="E16" s="86" t="inlineStr">
+        <is>
+          <t>unit-id</t>
+        </is>
+      </c>
       <c r="F16" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020015</t>
@@ -14795,17 +14917,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H16" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G16,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G16,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G16,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H16" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I16" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J16" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K16" s="110" t="inlineStr">
         <is>
@@ -14894,7 +15019,11 @@
       <c r="A17" s="117" t="n"/>
       <c r="C17" s="117" t="n"/>
       <c r="D17" s="119" t="n"/>
-      <c r="E17" s="86" t="n"/>
+      <c r="E17" s="86" t="inlineStr">
+        <is>
+          <t>roomnumberfm</t>
+        </is>
+      </c>
       <c r="F17" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020016</t>
@@ -14905,17 +15034,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H17" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G17,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I17" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G17,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G17,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H17" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I17" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J17" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K17" s="110" t="inlineStr">
         <is>
@@ -15004,7 +15136,11 @@
       <c r="A18" s="117" t="n"/>
       <c r="C18" s="117" t="n"/>
       <c r="D18" s="119" t="n"/>
-      <c r="E18" s="86" t="n"/>
+      <c r="E18" s="86" t="inlineStr">
+        <is>
+          <t>roomsignallabel</t>
+        </is>
+      </c>
       <c r="F18" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020017</t>
@@ -15015,17 +15151,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H18" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G18,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I18" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G18,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G18,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H18" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I18" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J18" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K18" s="110" t="inlineStr">
         <is>
@@ -15114,7 +15253,11 @@
       <c r="A19" s="117" t="n"/>
       <c r="C19" s="117" t="n"/>
       <c r="D19" s="119" t="n"/>
-      <c r="E19" s="86" t="n"/>
+      <c r="E19" s="86" t="inlineStr">
+        <is>
+          <t>cleaninggroup</t>
+        </is>
+      </c>
       <c r="F19" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020018</t>
@@ -15125,17 +15268,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H19" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G19,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I19" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G19,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G19,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H19" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I19" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J19" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K19" s="110" t="inlineStr">
         <is>
@@ -15224,7 +15370,11 @@
       <c r="A20" s="117" t="n"/>
       <c r="C20" s="117" t="n"/>
       <c r="D20" s="119" t="n"/>
-      <c r="E20" s="86" t="n"/>
+      <c r="E20" s="86" t="inlineStr">
+        <is>
+          <t>areaload</t>
+        </is>
+      </c>
       <c r="F20" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020019</t>
@@ -15235,17 +15385,20 @@
           <t>Physical characteristics</t>
         </is>
       </c>
-      <c r="H20" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G20,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G20,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G20,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H20" s="120" t="inlineStr">
+        <is>
+          <t>Physikalische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I20" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques physiques</t>
+        </is>
+      </c>
+      <c r="J20" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche fisiche</t>
+        </is>
       </c>
       <c r="K20" s="110" t="inlineStr">
         <is>
@@ -15334,7 +15487,11 @@
       <c r="A21" s="117" t="n"/>
       <c r="C21" s="117" t="n"/>
       <c r="D21" s="119" t="n"/>
-      <c r="E21" s="86" t="n"/>
+      <c r="E21" s="86" t="inlineStr">
+        <is>
+          <t>pointload</t>
+        </is>
+      </c>
       <c r="F21" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020020</t>
@@ -15345,17 +15502,20 @@
           <t>Physical characteristics</t>
         </is>
       </c>
-      <c r="H21" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G21,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I21" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G21,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G21,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H21" s="120" t="inlineStr">
+        <is>
+          <t>Physikalische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I21" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques physiques</t>
+        </is>
+      </c>
+      <c r="J21" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche fisiche</t>
+        </is>
       </c>
       <c r="K21" s="110" t="inlineStr">
         <is>
@@ -15444,7 +15604,11 @@
       <c r="A22" s="117" t="n"/>
       <c r="C22" s="117" t="n"/>
       <c r="D22" s="119" t="n"/>
-      <c r="E22" s="86" t="n"/>
+      <c r="E22" s="86" t="inlineStr">
+        <is>
+          <t>energyreferencearea</t>
+        </is>
+      </c>
       <c r="F22" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020021</t>
@@ -15455,17 +15619,20 @@
           <t>Physical characteristics</t>
         </is>
       </c>
-      <c r="H22" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G22,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G22,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G22,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H22" s="120" t="inlineStr">
+        <is>
+          <t>Physikalische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I22" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques physiques</t>
+        </is>
+      </c>
+      <c r="J22" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche fisiche</t>
+        </is>
       </c>
       <c r="K22" s="110" t="inlineStr">
         <is>
@@ -15554,7 +15721,11 @@
       <c r="A23" s="117" t="n"/>
       <c r="C23" s="117" t="n"/>
       <c r="D23" s="119" t="n"/>
-      <c r="E23" s="86" t="n"/>
+      <c r="E23" s="86" t="inlineStr">
+        <is>
+          <t>windowscleaningarea</t>
+        </is>
+      </c>
       <c r="F23" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020022</t>
@@ -15565,17 +15736,20 @@
           <t>Physical characteristics</t>
         </is>
       </c>
-      <c r="H23" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G23,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I23" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G23,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G23,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H23" s="120" t="inlineStr">
+        <is>
+          <t>Physikalische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I23" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques physiques</t>
+        </is>
+      </c>
+      <c r="J23" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche fisiche</t>
+        </is>
       </c>
       <c r="K23" s="110" t="inlineStr">
         <is>
@@ -15664,7 +15838,11 @@
       <c r="A24" s="117" t="n"/>
       <c r="C24" s="117" t="n"/>
       <c r="D24" s="119" t="n"/>
-      <c r="E24" s="86" t="n"/>
+      <c r="E24" s="86" t="inlineStr">
+        <is>
+          <t>windowsopenable</t>
+        </is>
+      </c>
       <c r="F24" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020023</t>
@@ -15675,17 +15853,20 @@
           <t>Performance characteristics</t>
         </is>
       </c>
-      <c r="H24" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G24,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I24" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G24,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G24,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H24" s="120" t="inlineStr">
+        <is>
+          <t>Leistungs- und Funktionskennwerte</t>
+        </is>
+      </c>
+      <c r="I24" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques de performance et de fonctionnement</t>
+        </is>
+      </c>
+      <c r="J24" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche prestazionali e funzionali</t>
+        </is>
       </c>
       <c r="K24" s="110" t="inlineStr">
         <is>
@@ -15774,7 +15955,11 @@
       <c r="A25" s="117" t="n"/>
       <c r="C25" s="117" t="n"/>
       <c r="D25" s="119" t="n"/>
-      <c r="E25" s="86" t="n"/>
+      <c r="E25" s="86" t="inlineStr">
+        <is>
+          <t>occupant</t>
+        </is>
+      </c>
       <c r="F25" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020024</t>
@@ -15785,17 +15970,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H25" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G25,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G25,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G25,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H25" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I25" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J25" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K25" s="110" t="inlineStr">
         <is>
@@ -15884,7 +16072,11 @@
       <c r="A26" s="117" t="n"/>
       <c r="C26" s="117" t="n"/>
       <c r="D26" s="119" t="n"/>
-      <c r="E26" s="86" t="n"/>
+      <c r="E26" s="86" t="inlineStr">
+        <is>
+          <t>shading</t>
+        </is>
+      </c>
       <c r="F26" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020025</t>
@@ -15895,17 +16087,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H26" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G26,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I26" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G26,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G26,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H26" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I26" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J26" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K26" s="110" t="inlineStr">
         <is>
@@ -15994,7 +16189,11 @@
       <c r="A27" s="117" t="n"/>
       <c r="C27" s="117" t="n"/>
       <c r="D27" s="119" t="n"/>
-      <c r="E27" s="86" t="n"/>
+      <c r="E27" s="86" t="inlineStr">
+        <is>
+          <t>ishumidified</t>
+        </is>
+      </c>
       <c r="F27" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020026</t>
@@ -16005,17 +16204,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H27" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G27,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I27" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G27,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J27" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G27,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H27" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I27" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J27" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K27" s="110" t="inlineStr">
         <is>
@@ -16104,7 +16306,11 @@
       <c r="A28" s="117" t="n"/>
       <c r="C28" s="117" t="n"/>
       <c r="D28" s="119" t="n"/>
-      <c r="E28" s="86" t="n"/>
+      <c r="E28" s="86" t="inlineStr">
+        <is>
+          <t>isdehumidified</t>
+        </is>
+      </c>
       <c r="F28" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020027</t>
@@ -16115,17 +16321,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H28" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G28,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I28" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G28,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G28,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H28" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I28" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J28" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K28" s="110" t="inlineStr">
         <is>
@@ -16214,7 +16423,11 @@
       <c r="A29" s="117" t="n"/>
       <c r="C29" s="117" t="n"/>
       <c r="D29" s="119" t="n"/>
-      <c r="E29" s="86" t="n"/>
+      <c r="E29" s="86" t="inlineStr">
+        <is>
+          <t>isrentable</t>
+        </is>
+      </c>
       <c r="F29" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020028</t>
@@ -16225,17 +16438,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H29" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G29,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I29" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G29,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J29" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G29,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H29" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I29" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J29" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K29" s="110" t="inlineStr">
         <is>
@@ -16328,7 +16544,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/IsExternal</t>
         </is>
       </c>
-      <c r="E30" s="86" t="n"/>
+      <c r="E30" s="86" t="inlineStr">
+        <is>
+          <t>isexternal</t>
+        </is>
+      </c>
       <c r="F30" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020029</t>
@@ -16339,17 +16559,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H30" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G30,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I30" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G30,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G30,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H30" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I30" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J30" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K30" s="110" t="inlineStr">
         <is>
@@ -16450,7 +16673,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyType</t>
         </is>
       </c>
-      <c r="E31" s="86" t="n"/>
+      <c r="E31" s="86" t="inlineStr">
+        <is>
+          <t>occupancytype</t>
+        </is>
+      </c>
       <c r="F31" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020030</t>
@@ -16461,17 +16688,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H31" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G31,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I31" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G31,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G31,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H31" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I31" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J31" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K31" s="110" t="inlineStr">
         <is>
@@ -16568,7 +16798,11 @@
       <c r="A32" s="117" t="n"/>
       <c r="C32" s="117" t="n"/>
       <c r="D32" s="119" t="n"/>
-      <c r="E32" s="86" t="n"/>
+      <c r="E32" s="86" t="inlineStr">
+        <is>
+          <t>minimumheadroom</t>
+        </is>
+      </c>
       <c r="F32" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020031</t>
@@ -16579,17 +16813,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H32" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G32,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G32,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G32,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H32" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I32" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J32" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K32" s="110" t="inlineStr">
         <is>
@@ -16686,7 +16923,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyNumberPeak</t>
         </is>
       </c>
-      <c r="E33" s="86" t="n"/>
+      <c r="E33" s="86" t="inlineStr">
+        <is>
+          <t>occupancynumberpeak</t>
+        </is>
+      </c>
       <c r="F33" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020032</t>
@@ -16697,17 +16938,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H33" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G33,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I33" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G33,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G33,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H33" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I33" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J33" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K33" s="110" t="inlineStr">
         <is>
@@ -16808,7 +17052,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyNumber</t>
         </is>
       </c>
-      <c r="E34" s="86" t="n"/>
+      <c r="E34" s="86" t="inlineStr">
+        <is>
+          <t>occupancynumber</t>
+        </is>
+      </c>
       <c r="F34" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020033</t>
@@ -16819,17 +17067,20 @@
           <t>Operating conditions and limits</t>
         </is>
       </c>
-      <c r="H34" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G34,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I34" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G34,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J34" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G34,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H34" s="120" t="inlineStr">
+        <is>
+          <t>Betriebsbedingungen und Grenzwerte</t>
+        </is>
+      </c>
+      <c r="I34" s="120" t="inlineStr">
+        <is>
+          <t>Conditions de fonctionnement et limites</t>
+        </is>
+      </c>
+      <c r="J34" s="120" t="inlineStr">
+        <is>
+          <t>Condizioni operative e limiti</t>
+        </is>
       </c>
       <c r="K34" s="110" t="inlineStr">
         <is>
@@ -16930,7 +17181,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/FloorCovering</t>
         </is>
       </c>
-      <c r="E35" s="86" t="n"/>
+      <c r="E35" s="86" t="inlineStr">
+        <is>
+          <t>floorcovering</t>
+        </is>
+      </c>
       <c r="F35" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020034</t>
@@ -16941,17 +17196,20 @@
           <t>Material and construction</t>
         </is>
       </c>
-      <c r="H35" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G35,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I35" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G35,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J35" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G35,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H35" s="120" t="inlineStr">
+        <is>
+          <t>Material und Aufbau</t>
+        </is>
+      </c>
+      <c r="I35" s="120" t="inlineStr">
+        <is>
+          <t>Matériau et constitution</t>
+        </is>
+      </c>
+      <c r="J35" s="120" t="inlineStr">
+        <is>
+          <t>Materiale e struttura</t>
+        </is>
       </c>
       <c r="K35" s="110" t="inlineStr">
         <is>
@@ -17052,7 +17310,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/WallCovering</t>
         </is>
       </c>
-      <c r="E36" s="86" t="n"/>
+      <c r="E36" s="86" t="inlineStr">
+        <is>
+          <t>wallcovering</t>
+        </is>
+      </c>
       <c r="F36" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020035</t>
@@ -17063,17 +17325,20 @@
           <t>Manufacturer and product information</t>
         </is>
       </c>
-      <c r="H36" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G36,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I36" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G36,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G36,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H36" s="120" t="inlineStr">
+        <is>
+          <t>Hersteller- und Produktinformationen</t>
+        </is>
+      </c>
+      <c r="I36" s="120" t="inlineStr">
+        <is>
+          <t>Informations sur le fabricant et le produit</t>
+        </is>
+      </c>
+      <c r="J36" s="120" t="inlineStr">
+        <is>
+          <t>Informazioni sul produttore e sul prodotto</t>
+        </is>
       </c>
       <c r="K36" s="110" t="inlineStr">
         <is>
@@ -17174,7 +17439,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/CeilingCovering</t>
         </is>
       </c>
-      <c r="E37" s="86" t="n"/>
+      <c r="E37" s="86" t="inlineStr">
+        <is>
+          <t>ceilingcovering</t>
+        </is>
+      </c>
       <c r="F37" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020036</t>
@@ -17185,17 +17454,20 @@
           <t>Material and construction</t>
         </is>
       </c>
-      <c r="H37" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G37,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I37" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G37,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J37" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G37,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H37" s="120" t="inlineStr">
+        <is>
+          <t>Material und Aufbau</t>
+        </is>
+      </c>
+      <c r="I37" s="120" t="inlineStr">
+        <is>
+          <t>Matériau et constitution</t>
+        </is>
+      </c>
+      <c r="J37" s="120" t="inlineStr">
+        <is>
+          <t>Materiale e struttura</t>
+        </is>
       </c>
       <c r="K37" s="110" t="inlineStr">
         <is>
@@ -17296,7 +17568,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NaturalVentilation</t>
         </is>
       </c>
-      <c r="E38" s="86" t="n"/>
+      <c r="E38" s="86" t="inlineStr">
+        <is>
+          <t>naturalventilation</t>
+        </is>
+      </c>
       <c r="F38" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020037</t>
@@ -17307,17 +17583,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H38" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G38,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I38" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G38,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J38" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G38,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H38" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I38" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J38" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K38" s="110" t="inlineStr">
         <is>
@@ -17418,7 +17697,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NaturalVentilationRate</t>
         </is>
       </c>
-      <c r="E39" s="86" t="n"/>
+      <c r="E39" s="86" t="inlineStr">
+        <is>
+          <t>naturalventilationrate</t>
+        </is>
+      </c>
       <c r="F39" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020038</t>
@@ -17429,17 +17712,20 @@
           <t>Hydraulic / flow characteristics</t>
         </is>
       </c>
-      <c r="H39" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G39,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I39" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G39,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G39,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H39" s="120" t="inlineStr">
+        <is>
+          <t>Hydraulische / strömungstechnische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I39" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques hydrauliques / d’écoulement</t>
+        </is>
+      </c>
+      <c r="J39" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche idrauliche / di flusso</t>
+        </is>
       </c>
       <c r="K39" s="110" t="inlineStr">
         <is>
@@ -17540,7 +17826,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/MechanicalVentilation</t>
         </is>
       </c>
-      <c r="E40" s="86" t="n"/>
+      <c r="E40" s="86" t="inlineStr">
+        <is>
+          <t>mechanicalventilation</t>
+        </is>
+      </c>
       <c r="F40" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020039</t>
@@ -17551,17 +17841,20 @@
           <t>Performance characteristics</t>
         </is>
       </c>
-      <c r="H40" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G40,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I40" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G40,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J40" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G40,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H40" s="120" t="inlineStr">
+        <is>
+          <t>Leistungs- und Funktionskennwerte</t>
+        </is>
+      </c>
+      <c r="I40" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques de performance et de fonctionnement</t>
+        </is>
+      </c>
+      <c r="J40" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche prestazionali e funzionali</t>
+        </is>
       </c>
       <c r="K40" s="110" t="inlineStr">
         <is>
@@ -17662,7 +17955,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/MechanicalVentilationRate</t>
         </is>
       </c>
-      <c r="E41" s="86" t="n"/>
+      <c r="E41" s="86" t="inlineStr">
+        <is>
+          <t>mechanicalventilationrate</t>
+        </is>
+      </c>
       <c r="F41" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020040</t>
@@ -17673,17 +17970,20 @@
           <t>Hydraulic / flow characteristics</t>
         </is>
       </c>
-      <c r="H41" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G41,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I41" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G41,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J41" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G41,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H41" s="120" t="inlineStr">
+        <is>
+          <t>Hydraulische / strömungstechnische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I41" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques hydrauliques / d’écoulement</t>
+        </is>
+      </c>
+      <c r="J41" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche idrauliche / di flusso</t>
+        </is>
       </c>
       <c r="K41" s="110" t="inlineStr">
         <is>
@@ -17784,7 +18084,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/AirConditioning</t>
         </is>
       </c>
-      <c r="E42" s="86" t="n"/>
+      <c r="E42" s="86" t="inlineStr">
+        <is>
+          <t>airconditioning</t>
+        </is>
+      </c>
       <c r="F42" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020041</t>
@@ -17795,17 +18099,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H42" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G42,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I42" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G42,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J42" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G42,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H42" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I42" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J42" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K42" s="110" t="inlineStr">
         <is>
@@ -17906,7 +18213,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/TemperatureSetPoint</t>
         </is>
       </c>
-      <c r="E43" s="86" t="n"/>
+      <c r="E43" s="86" t="inlineStr">
+        <is>
+          <t>temperaturesetpoint</t>
+        </is>
+      </c>
       <c r="F43" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020042</t>
@@ -17917,17 +18228,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H43" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G43,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I43" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G43,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J43" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G43,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H43" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I43" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J43" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K43" s="110" t="inlineStr">
         <is>
@@ -18028,7 +18342,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/HumiditySetPoint</t>
         </is>
       </c>
-      <c r="E44" s="86" t="n"/>
+      <c r="E44" s="86" t="inlineStr">
+        <is>
+          <t>humiditysetpoint</t>
+        </is>
+      </c>
       <c r="F44" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020043</t>
@@ -18039,17 +18357,20 @@
           <t>Thermal characteristics</t>
         </is>
       </c>
-      <c r="H44" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G44,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I44" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G44,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J44" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G44,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H44" s="120" t="inlineStr">
+        <is>
+          <t>Thermische Kennwerte</t>
+        </is>
+      </c>
+      <c r="I44" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques thermiques</t>
+        </is>
+      </c>
+      <c r="J44" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche termiche</t>
+        </is>
       </c>
       <c r="K44" s="110" t="inlineStr">
         <is>
@@ -18150,7 +18471,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/FireExit</t>
         </is>
       </c>
-      <c r="E45" s="86" t="n"/>
+      <c r="E45" s="86" t="inlineStr">
+        <is>
+          <t>fireexit</t>
+        </is>
+      </c>
       <c r="F45" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020044</t>
@@ -18161,17 +18486,20 @@
           <t>Safety and protection characteristics</t>
         </is>
       </c>
-      <c r="H45" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G45,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I45" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G45,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J45" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G45,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H45" s="120" t="inlineStr">
+        <is>
+          <t>Sicherheits- und Schutzmerkmale</t>
+        </is>
+      </c>
+      <c r="I45" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques de sécurité et de protection</t>
+        </is>
+      </c>
+      <c r="J45" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche di sicurezza e protezione</t>
+        </is>
       </c>
       <c r="K45" s="110" t="inlineStr">
         <is>
@@ -18272,7 +18600,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/GrossFloorArea</t>
         </is>
       </c>
-      <c r="E46" s="86" t="n"/>
+      <c r="E46" s="86" t="inlineStr">
+        <is>
+          <t>grossfloorarea</t>
+        </is>
+      </c>
       <c r="F46" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020045</t>
@@ -18283,17 +18615,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H46" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G46,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I46" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G46,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J46" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G46,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H46" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I46" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J46" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K46" s="110" t="inlineStr">
         <is>
@@ -18394,7 +18729,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/GrossVolume</t>
         </is>
       </c>
-      <c r="E47" s="86" t="n"/>
+      <c r="E47" s="86" t="inlineStr">
+        <is>
+          <t>grossvolume</t>
+        </is>
+      </c>
       <c r="F47" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020046</t>
@@ -18405,17 +18744,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H47" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G47,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I47" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G47,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G47,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H47" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I47" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J47" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K47" s="110" t="inlineStr">
         <is>
@@ -18516,7 +18858,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NetFloorArea</t>
         </is>
       </c>
-      <c r="E48" s="86" t="n"/>
+      <c r="E48" s="86" t="inlineStr">
+        <is>
+          <t>netfloorarea</t>
+        </is>
+      </c>
       <c r="F48" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020047</t>
@@ -18527,17 +18873,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H48" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G48,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I48" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G48,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J48" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G48,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H48" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I48" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J48" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K48" s="110" t="inlineStr">
         <is>
@@ -18638,7 +18987,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NetVolume</t>
         </is>
       </c>
-      <c r="E49" s="86" t="n"/>
+      <c r="E49" s="86" t="inlineStr">
+        <is>
+          <t>netvolume</t>
+        </is>
+      </c>
       <c r="F49" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020048</t>
@@ -18649,17 +19002,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H49" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G49,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I49" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G49,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J49" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G49,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H49" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I49" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J49" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K49" s="110" t="inlineStr">
         <is>
@@ -18756,7 +19112,11 @@
       <c r="A50" s="117" t="n"/>
       <c r="C50" s="117" t="n"/>
       <c r="D50" s="119" t="n"/>
-      <c r="E50" s="86" t="n"/>
+      <c r="E50" s="86" t="inlineStr">
+        <is>
+          <t>netwallarea</t>
+        </is>
+      </c>
       <c r="F50" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020049</t>
@@ -18767,17 +19127,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H50" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G50,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I50" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G50,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J50" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G50,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H50" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I50" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J50" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K50" s="110" t="inlineStr">
         <is>
@@ -18874,7 +19237,11 @@
           <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/Height</t>
         </is>
       </c>
-      <c r="E51" s="86" t="n"/>
+      <c r="E51" s="86" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
       <c r="F51" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020050</t>
@@ -18885,17 +19252,20 @@
           <t>Geometric characteristics</t>
         </is>
       </c>
-      <c r="H51" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G51,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G51,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J51" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G51,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H51" s="120" t="inlineStr">
+        <is>
+          <t>Geometrische Eigenschaften</t>
+        </is>
+      </c>
+      <c r="I51" s="120" t="inlineStr">
+        <is>
+          <t>Caractéristiques géométriques</t>
+        </is>
+      </c>
+      <c r="J51" s="120" t="inlineStr">
+        <is>
+          <t>Caratteristiche geometriche</t>
+        </is>
       </c>
       <c r="K51" s="110" t="inlineStr">
         <is>
@@ -18992,7 +19362,11 @@
       <c r="A52" s="117" t="n"/>
       <c r="C52" s="117" t="n"/>
       <c r="D52" s="119" t="n"/>
-      <c r="E52" s="86" t="n"/>
+      <c r="E52" s="86" t="inlineStr">
+        <is>
+          <t>aboveground</t>
+        </is>
+      </c>
       <c r="F52" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020051</t>
@@ -19003,17 +19377,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H52" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G52,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I52" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G52,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J52" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G52,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H52" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I52" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J52" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K52" s="110" t="inlineStr">
         <is>
@@ -19098,7 +19475,11 @@
       <c r="A53" s="117" t="n"/>
       <c r="C53" s="117" t="n"/>
       <c r="D53" s="119" t="n"/>
-      <c r="E53" s="86" t="n"/>
+      <c r="E53" s="86" t="inlineStr">
+        <is>
+          <t>costzone</t>
+        </is>
+      </c>
       <c r="F53" s="91" t="inlineStr">
         <is>
           <t>IFMA_P_31020052</t>
@@ -19109,17 +19490,20 @@
           <t>Identification and classification</t>
         </is>
       </c>
-      <c r="H53" s="120">
-        <f>IFERROR(INDEX(Rules!$F:$F,MATCH(G53,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I53" s="120">
-        <f>IFERROR(INDEX(Rules!$G:$G,MATCH(G53,Rules!$E:$E,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J53" s="120">
-        <f>IFERROR(INDEX(Rules!$H:$H,MATCH(G53,Rules!$E:$E,0)),"")</f>
-        <v/>
+      <c r="H53" s="120" t="inlineStr">
+        <is>
+          <t>Identifikation und Klassifikation</t>
+        </is>
+      </c>
+      <c r="I53" s="120" t="inlineStr">
+        <is>
+          <t>Identification et classification</t>
+        </is>
+      </c>
+      <c r="J53" s="120" t="inlineStr">
+        <is>
+          <t>Identificazione e classificazione</t>
+        </is>
       </c>
       <c r="K53" s="110" t="inlineStr">
         <is>
@@ -21297,7 +21681,11 @@
       <c r="B7" s="103" t="n"/>
       <c r="C7" s="103" t="n"/>
       <c r="D7" s="235" t="n"/>
-      <c r="E7" s="86" t="n"/>
+      <c r="E7" s="86" t="inlineStr">
+        <is>
+          <t>predefinedtype_enum</t>
+        </is>
+      </c>
       <c r="F7" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030000</t>
@@ -21376,7 +21764,11 @@
       <c r="B8" s="103" t="n"/>
       <c r="C8" s="103" t="n"/>
       <c r="D8" s="235" t="n"/>
-      <c r="E8" s="86" t="n"/>
+      <c r="E8" s="86" t="inlineStr">
+        <is>
+          <t>objecttype_enum</t>
+        </is>
+      </c>
       <c r="F8" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030001</t>
@@ -21455,7 +21847,11 @@
       <c r="B9" s="103" t="n"/>
       <c r="C9" s="103" t="n"/>
       <c r="D9" s="235" t="n"/>
-      <c r="E9" s="86" t="n"/>
+      <c r="E9" s="86" t="inlineStr">
+        <is>
+          <t>area_type_sia_416_code_enum</t>
+        </is>
+      </c>
       <c r="F9" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030004</t>
@@ -21534,7 +21930,11 @@
       <c r="B10" s="103" t="n"/>
       <c r="C10" s="103" t="n"/>
       <c r="D10" s="235" t="n"/>
-      <c r="E10" s="86" t="n"/>
+      <c r="E10" s="86" t="inlineStr">
+        <is>
+          <t>room_designation_sia_380_label_enum</t>
+        </is>
+      </c>
       <c r="F10" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030007</t>
@@ -21613,7 +22013,11 @@
       <c r="B11" s="103" t="n"/>
       <c r="C11" s="103" t="n"/>
       <c r="D11" s="235" t="n"/>
-      <c r="E11" s="86" t="n"/>
+      <c r="E11" s="86" t="inlineStr">
+        <is>
+          <t>room_usage_sia_2024_code_enum</t>
+        </is>
+      </c>
       <c r="F11" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030008</t>
@@ -21688,7 +22092,11 @@
       <c r="B12" s="103" t="n"/>
       <c r="C12" s="103" t="n"/>
       <c r="D12" s="235" t="n"/>
-      <c r="E12" s="86" t="n"/>
+      <c r="E12" s="86" t="inlineStr">
+        <is>
+          <t>area_type_d0165_code_enum</t>
+        </is>
+      </c>
       <c r="F12" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030010</t>
@@ -21763,7 +22171,11 @@
       <c r="B13" s="103" t="n"/>
       <c r="C13" s="103" t="n"/>
       <c r="D13" s="235" t="n"/>
-      <c r="E13" s="86" t="n"/>
+      <c r="E13" s="86" t="inlineStr">
+        <is>
+          <t>energy_reference_area_enum</t>
+        </is>
+      </c>
       <c r="F13" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030021</t>
@@ -21842,7 +22254,11 @@
       <c r="B14" s="103" t="n"/>
       <c r="C14" s="103" t="n"/>
       <c r="D14" s="235" t="n"/>
-      <c r="E14" s="86" t="n"/>
+      <c r="E14" s="86" t="inlineStr">
+        <is>
+          <t>window_openable_enum</t>
+        </is>
+      </c>
       <c r="F14" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030023</t>
@@ -21921,7 +22337,11 @@
       <c r="B15" s="103" t="n"/>
       <c r="C15" s="103" t="n"/>
       <c r="D15" s="235" t="n"/>
-      <c r="E15" s="86" t="n"/>
+      <c r="E15" s="86" t="inlineStr">
+        <is>
+          <t>solar_shading_enum</t>
+        </is>
+      </c>
       <c r="F15" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030025</t>
@@ -22000,7 +22420,11 @@
       <c r="B16" s="103" t="n"/>
       <c r="C16" s="103" t="n"/>
       <c r="D16" s="235" t="n"/>
-      <c r="E16" s="86" t="n"/>
+      <c r="E16" s="86" t="inlineStr">
+        <is>
+          <t>humidified_enum</t>
+        </is>
+      </c>
       <c r="F16" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030026</t>
@@ -22077,7 +22501,11 @@
     <row r="17" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B17" s="103" t="n"/>
       <c r="D17" s="235" t="n"/>
-      <c r="E17" s="86" t="n"/>
+      <c r="E17" s="86" t="inlineStr">
+        <is>
+          <t>dehumidified_enum</t>
+        </is>
+      </c>
       <c r="F17" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030027</t>
@@ -22153,7 +22581,11 @@
     <row r="18" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B18" s="103" t="n"/>
       <c r="D18" s="235" t="n"/>
-      <c r="E18" s="86" t="n"/>
+      <c r="E18" s="86" t="inlineStr">
+        <is>
+          <t>rentable_enum</t>
+        </is>
+      </c>
       <c r="F18" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030028</t>
@@ -22229,7 +22661,11 @@
     <row r="19" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B19" s="103" t="n"/>
       <c r="D19" s="235" t="n"/>
-      <c r="E19" s="86" t="n"/>
+      <c r="E19" s="86" t="inlineStr">
+        <is>
+          <t>external_space_enum</t>
+        </is>
+      </c>
       <c r="F19" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030029</t>
@@ -22305,7 +22741,11 @@
     <row r="20" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B20" s="103" t="n"/>
       <c r="D20" s="235" t="n"/>
-      <c r="E20" s="86" t="n"/>
+      <c r="E20" s="86" t="inlineStr">
+        <is>
+          <t>natural_ventilation_enum</t>
+        </is>
+      </c>
       <c r="F20" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030037</t>
@@ -22381,7 +22821,11 @@
     <row r="21" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B21" s="103" t="n"/>
       <c r="D21" s="235" t="n"/>
-      <c r="E21" s="86" t="n"/>
+      <c r="E21" s="86" t="inlineStr">
+        <is>
+          <t>mechanical_ventilation_enum</t>
+        </is>
+      </c>
       <c r="F21" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030039</t>
@@ -22457,7 +22901,11 @@
     <row r="22" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B22" s="103" t="n"/>
       <c r="D22" s="235" t="n"/>
-      <c r="E22" s="86" t="n"/>
+      <c r="E22" s="86" t="inlineStr">
+        <is>
+          <t>air_conditioning_enum</t>
+        </is>
+      </c>
       <c r="F22" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030041</t>
@@ -22533,7 +22981,11 @@
     <row r="23" ht="14.25" customFormat="1" customHeight="1" s="237">
       <c r="B23" s="103" t="n"/>
       <c r="D23" s="235" t="n"/>
-      <c r="E23" s="86" t="n"/>
+      <c r="E23" s="86" t="inlineStr">
+        <is>
+          <t>fire_exit_enum</t>
+        </is>
+      </c>
       <c r="F23" s="91" t="inlineStr">
         <is>
           <t>IFMA_V_31030044</t>
@@ -23225,7 +23677,11 @@
     </row>
     <row r="7" ht="25.5" customFormat="1" customHeight="1" s="104">
       <c r="D7" s="105" t="n"/>
-      <c r="E7" s="86" t="n"/>
+      <c r="E7" s="86" t="inlineStr">
+        <is>
+          <t>sn-504-416-areas-and-volumes-of-buildings</t>
+        </is>
+      </c>
       <c r="F7" s="91" t="inlineStr">
         <is>
           <t>IFMA_D_31040000</t>
@@ -24084,7 +24540,11 @@
     <row r="7" ht="102" customFormat="1" customHeight="1" s="85">
       <c r="A7" s="84" t="n"/>
       <c r="C7" s="84" t="n"/>
-      <c r="D7" s="105" t="n"/>
+      <c r="D7" s="105" t="inlineStr">
+        <is>
+          <t>ifma-areamgmt</t>
+        </is>
+      </c>
       <c r="E7" s="86" t="n"/>
       <c r="F7" s="87" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Align SchemaForge pipeline with NatDD core schema
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_AreaMgmt_v0.5.0.xlsx
+++ b/templates/Strukturvorlage_AreaMgmt_v0.5.0.xlsx
@@ -24892,7 +24892,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col width="40.7109375" customWidth="1" style="41" min="1" max="1"/>
-    <col width="1.7109375" customWidth="1" style="41" min="2" max="2"/>
+    <col width="28" customWidth="1" style="41" min="2" max="2"/>
     <col width="21.85546875" customWidth="1" style="50" min="3" max="3"/>
     <col width="1.7109375" customWidth="1" style="41" min="4" max="4"/>
     <col width="6.42578125" bestFit="1" customWidth="1" style="50" min="5" max="5"/>
@@ -24916,6 +24916,11 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.65" customHeight="1" s="249">
+      <c r="B1" s="47" t="inlineStr">
+        <is>
+          <t>Data Templates</t>
+        </is>
+      </c>
       <c r="C1" s="47" t="inlineStr">
         <is>
           <t>GoP</t>
@@ -24984,7 +24989,11 @@
       <c r="BG1" s="47" t="n"/>
     </row>
     <row r="2" ht="318.75" customFormat="1" customHeight="1" s="42">
-      <c r="B2" s="41" t="n"/>
+      <c r="B2" s="48" t="inlineStr">
+        <is>
+          <t>DataTemplate-ID</t>
+        </is>
+      </c>
       <c r="C2" s="48" t="inlineStr">
         <is>
           <t>GoP - Designation/Bezeichnung/Désignation/Designazione</t>
@@ -25245,6 +25254,11 @@
           <t>Classes</t>
         </is>
       </c>
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Stable identity</t>
+        </is>
+      </c>
       <c r="C3" s="41" t="n"/>
       <c r="E3" s="41" t="n"/>
       <c r="BC3" s="41" t="n"/>
@@ -25255,7 +25269,11 @@
           <t>Class - Designation/Bezeichnung/Désignation/Designazione</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>Repeat the same ID across rows to attach 0..n GroupOfProperties</t>
+        </is>
+      </c>
       <c r="C4" s="52" t="n"/>
       <c r="D4" s="45" t="n"/>
       <c r="E4" s="52" t="n"/>
@@ -25313,7 +25331,11 @@
         <f>Classes!P7</f>
         <v/>
       </c>
-      <c r="B5" s="41" t="n"/>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>geschossebene-dt</t>
+        </is>
+      </c>
       <c r="C5" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -25386,7 +25408,11 @@
         <f>Classes!P8</f>
         <v/>
       </c>
-      <c r="B6" s="41" t="n"/>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>grundstueckflaeche-dt</t>
+        </is>
+      </c>
       <c r="C6" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -25461,7 +25487,11 @@
         <f>Classes!P9</f>
         <v/>
       </c>
-      <c r="B7" s="41" t="n"/>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>umgebungsflaeche-dt</t>
+        </is>
+      </c>
       <c r="C7" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -25565,7 +25595,11 @@
         <f>Classes!P10</f>
         <v/>
       </c>
-      <c r="B8" s="41" t="n"/>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>geschossvolumen-dt</t>
+        </is>
+      </c>
       <c r="C8" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -25665,7 +25699,11 @@
         <f>Classes!P11</f>
         <v/>
       </c>
-      <c r="B9" s="41" t="n"/>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>nettogeschossflaeche-dt</t>
+        </is>
+      </c>
       <c r="C9" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -25905,7 +25943,11 @@
         <f>Classes!P12</f>
         <v/>
       </c>
-      <c r="B10" s="41" t="n"/>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>aussen-nettogeschossflaeche-dt</t>
+        </is>
+      </c>
       <c r="C10" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -26029,7 +26071,11 @@
         <f>Classes!P13</f>
         <v/>
       </c>
-      <c r="B11" s="41" t="n"/>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>stellplatz-dt</t>
+        </is>
+      </c>
       <c r="C11" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>
@@ -26125,7 +26171,11 @@
         <f>Classes!P14</f>
         <v/>
       </c>
-      <c r="B12" s="41" t="n"/>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>vermietbare-flaeche-dt</t>
+        </is>
+      </c>
       <c r="C12" s="46" t="inlineStr">
         <is>
           <t>IFMA_AreaMgmt</t>

</xml_diff>